<commit_message>
Correct Secured Exit Notes coupon to 10% per RSA Term Sheet
RSA Term Sheet ¶109 specifies 10% cash coupon on the $420M Secured
Exit Notes due 2031 (not 9%). Corrected rate now reconciles to the
$101M of 2027 cash interest disclosed in the Projections.

https://claude.ai/code/session_01MHrifSmTXze7ixJ3nQDz5f
</commit_message>
<xml_diff>
--- a/Q7_Sustainable_Cash_Interest.xlsx
+++ b/Q7_Sustainable_Cash_Interest.xlsx
@@ -703,7 +703,7 @@
         <v/>
       </c>
       <c r="C14" s="9" t="n">
-        <v>0.09</v>
+        <v>0.1</v>
       </c>
       <c r="D14" s="8">
         <f>B14*C14</f>
@@ -716,7 +716,7 @@
       </c>
       <c r="F14" s="10" t="inlineStr">
         <is>
-          <t>Disc Stmt Ex B</t>
+          <t>RSA Term Sheet ¶109 (10% cash)</t>
         </is>
       </c>
     </row>

</xml_diff>